<commit_message>
fix: starch content load function
</commit_message>
<xml_diff>
--- a/biorefineries/isobutanol/analyses/full/parameter_distributions/parameter-distributions_corn_IBO_EtOH_A.xlsx
+++ b/biorefineries/isobutanol/analyses/full/parameter_distributions/parameter-distributions_corn_IBO_EtOH_A.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\saran\Documents\Academia\repository_clones\Bioindustrial-Park\biorefineries\isobutanol\analyses\full\parameter_distributions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6EDC3A7-2A4F-4EA9-B5B1-0964BDF6A7DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8EEB212C-82B1-4CCC-BF55-6EB86BD9AD25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="2490" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -518,12 +518,6 @@
     <t>Feedstock starch content</t>
   </si>
   <si>
-    <t>kg/kg-water</t>
-  </si>
-  <si>
-    <t>feedstock.imass['Starch'] =x * feedstock.imass['Water']</t>
-  </si>
-  <si>
     <t>Aeration rate safety factor</t>
   </si>
   <si>
@@ -534,6 +528,12 @@
   </si>
   <si>
     <t>DDGS unit price (sale)</t>
+  </si>
+  <si>
+    <t>kg/dry-kg</t>
+  </si>
+  <si>
+    <t>fixed_F_mass = feedstock.F_mass; feedstock.imass['Starch'] = x * (fixed_F_mass - feedstock.imass['Water']); feedstock.F_mass = fixed_F_mass</t>
   </si>
 </sst>
 </file>
@@ -1244,7 +1244,7 @@
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A11" s="4" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="B11" s="4" t="s">
         <v>7</v>
@@ -1419,29 +1419,29 @@
         <v>21</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="E16" s="3">
-        <v>4.08</v>
+        <v>0.72</v>
       </c>
       <c r="F16" s="3" t="s">
         <v>27</v>
       </c>
       <c r="G16" s="3">
         <f>0.8*H16</f>
-        <v>3.2640000000000002</v>
+        <v>0.57599999999999996</v>
       </c>
       <c r="H16" s="3">
         <f>E16</f>
-        <v>4.08</v>
+        <v>0.72</v>
       </c>
       <c r="I16" s="3">
         <f>1.2*H16</f>
-        <v>4.8959999999999999</v>
+        <v>0.86399999999999999</v>
       </c>
       <c r="J16" s="3"/>
       <c r="K16" s="3" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.35">
@@ -1482,10 +1482,10 @@
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A18" s="3" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="C18" s="3" t="s">
         <v>21</v>
@@ -1508,7 +1508,7 @@
       </c>
       <c r="J18" s="3"/>
       <c r="K18" s="3" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
default to 80-120% uniform for uncertainty in raw material purchase prices
</commit_message>
<xml_diff>
--- a/biorefineries/isobutanol/analyses/full/parameter_distributions/parameter-distributions_corn_IBO_EtOH_A.xlsx
+++ b/biorefineries/isobutanol/analyses/full/parameter_distributions/parameter-distributions_corn_IBO_EtOH_A.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\saran\Documents\Academia\repository_clones\Bioindustrial-Park\biorefineries\isobutanol\analyses\full\parameter_distributions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8EEB212C-82B1-4CCC-BF55-6EB86BD9AD25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D34303BB-A1B5-46C8-9072-A86A70FA1727}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1325,19 +1325,19 @@
         <v>0.10355</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>27</v>
+        <v>18</v>
       </c>
       <c r="G13" s="6">
-        <f>E13*0.9</f>
-        <v>9.3195E-2</v>
+        <f>E13*0.8</f>
+        <v>8.2840000000000011E-2</v>
       </c>
       <c r="H13" s="6">
         <f>E13</f>
         <v>0.10355</v>
       </c>
       <c r="I13" s="6">
-        <f>E13*1.1</f>
-        <v>0.11390500000000001</v>
+        <f>E13*1.2</f>
+        <v>0.12426</v>
       </c>
       <c r="J13" s="6"/>
       <c r="K13" s="6" t="s">

</xml_diff>

<commit_message>
update for nsk reset call refactor
</commit_message>
<xml_diff>
--- a/biorefineries/isobutanol/analyses/full/parameter_distributions/parameter-distributions_corn_IBO_EtOH_A.xlsx
+++ b/biorefineries/isobutanol/analyses/full/parameter_distributions/parameter-distributions_corn_IBO_EtOH_A.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\saran\Documents\Academia\repository_clones\Bioindustrial-Park\biorefineries\isobutanol\analyses\full\parameter_distributions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D34303BB-A1B5-46C8-9072-A86A70FA1727}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11D9513E-CA76-42FF-9D18-367610097181}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1331,10 +1331,7 @@
         <f>E13*0.8</f>
         <v>8.2840000000000011E-2</v>
       </c>
-      <c r="H13" s="6">
-        <f>E13</f>
-        <v>0.10355</v>
-      </c>
+      <c r="H13" s="6"/>
       <c r="I13" s="6">
         <f>E13*1.2</f>
         <v>0.12426</v>

</xml_diff>

<commit_message>
update for nskinetics rename of kinetic_reaction_system to nsk_kinetic_model
Rename attribute references across system, utils, analyses, and the
scenario A/B parameter-distributions xlsx setter statements; matches
nskinetics a0f7c11. Smoke tests validated (A ~0.745, B ~0.991, 2x each).
</commit_message>
<xml_diff>
--- a/biorefineries/isobutanol/analyses/full/parameter_distributions/parameter-distributions_corn_IBO_EtOH_A.xlsx
+++ b/biorefineries/isobutanol/analyses/full/parameter_distributions/parameter-distributions_corn_IBO_EtOH_A.xlsx
@@ -206,31 +206,31 @@
     <t>V514.tau = x</t>
   </si>
   <si>
-    <t>V406.kinetic_reaction_system._te.k_2 = x</t>
-  </si>
-  <si>
-    <t>V406.kinetic_reaction_system._te.k_1e = x</t>
-  </si>
-  <si>
-    <t>V406.kinetic_reaction_system._te.k_1h = x</t>
-  </si>
-  <si>
-    <t>V406.kinetic_reaction_system._te.k_1ie = x</t>
-  </si>
-  <si>
-    <t>V406.kinetic_reaction_system._te.k_1ia = x</t>
-  </si>
-  <si>
-    <t>V406.kinetic_reaction_system._te.k_1ii = x</t>
-  </si>
-  <si>
-    <t>V406.kinetic_reaction_system._te.k_1l = x</t>
-  </si>
-  <si>
-    <t>V406.kinetic_reaction_system._te.k_3 = x</t>
-  </si>
-  <si>
-    <t>V406.kinetic_reaction_system._te.k_4 = x</t>
+    <t>V406.nsk_kinetic_model._te.k_2 = x</t>
+  </si>
+  <si>
+    <t>V406.nsk_kinetic_model._te.k_1e = x</t>
+  </si>
+  <si>
+    <t>V406.nsk_kinetic_model._te.k_1h = x</t>
+  </si>
+  <si>
+    <t>V406.nsk_kinetic_model._te.k_1ie = x</t>
+  </si>
+  <si>
+    <t>V406.nsk_kinetic_model._te.k_1ia = x</t>
+  </si>
+  <si>
+    <t>V406.nsk_kinetic_model._te.k_1ii = x</t>
+  </si>
+  <si>
+    <t>V406.nsk_kinetic_model._te.k_1l = x</t>
+  </si>
+  <si>
+    <t>V406.nsk_kinetic_model._te.k_3 = x</t>
+  </si>
+  <si>
+    <t>V406.nsk_kinetic_model._te.k_4 = x</t>
   </si>
   <si>
     <t>g_per_l_per_h</t>
@@ -242,55 +242,55 @@
     <t>g_per_l</t>
   </si>
   <si>
-    <t>V406.kinetic_reaction_system._te.k_4ie = x</t>
-  </si>
-  <si>
-    <t>V406.kinetic_reaction_system._te.k_4ia = x</t>
-  </si>
-  <si>
-    <t>V406.kinetic_reaction_system._te.k_4ii = x</t>
-  </si>
-  <si>
-    <t>V406.kinetic_reaction_system._te.k_5 = x</t>
-  </si>
-  <si>
-    <t>V406.kinetic_reaction_system._te.k_5e = x</t>
-  </si>
-  <si>
-    <t>V406.kinetic_reaction_system._te.k_6 = x</t>
-  </si>
-  <si>
-    <t>V406.kinetic_reaction_system._te.k_6r = x</t>
-  </si>
-  <si>
-    <t>V406.kinetic_reaction_system._te.k_7 = x</t>
-  </si>
-  <si>
-    <t>V406.kinetic_reaction_system._te.k_7ie = x</t>
-  </si>
-  <si>
-    <t>V406.kinetic_reaction_system._te.k_7ia = x</t>
-  </si>
-  <si>
-    <t>V406.kinetic_reaction_system._te.k_7ii = x</t>
-  </si>
-  <si>
-    <t>V406.kinetic_reaction_system._te.k_8 = x</t>
-  </si>
-  <si>
-    <t>V406.kinetic_reaction_system._te.k_9 = x</t>
-  </si>
-  <si>
-    <t>V406.kinetic_reaction_system._te.k_9e = x</t>
-  </si>
-  <si>
-    <t>V406.kinetic_reaction_system._te.k_9c = x</t>
-  </si>
-  <si>
-    <t>V406.kinetic_reaction_system._te.k_10 = x</t>
-  </si>
-  <si>
-    <t>V406.kinetic_reaction_system._te.k_11 = x</t>
+    <t>V406.nsk_kinetic_model._te.k_4ie = x</t>
+  </si>
+  <si>
+    <t>V406.nsk_kinetic_model._te.k_4ia = x</t>
+  </si>
+  <si>
+    <t>V406.nsk_kinetic_model._te.k_4ii = x</t>
+  </si>
+  <si>
+    <t>V406.nsk_kinetic_model._te.k_5 = x</t>
+  </si>
+  <si>
+    <t>V406.nsk_kinetic_model._te.k_5e = x</t>
+  </si>
+  <si>
+    <t>V406.nsk_kinetic_model._te.k_6 = x</t>
+  </si>
+  <si>
+    <t>V406.nsk_kinetic_model._te.k_6r = x</t>
+  </si>
+  <si>
+    <t>V406.nsk_kinetic_model._te.k_7 = x</t>
+  </si>
+  <si>
+    <t>V406.nsk_kinetic_model._te.k_7ie = x</t>
+  </si>
+  <si>
+    <t>V406.nsk_kinetic_model._te.k_7ia = x</t>
+  </si>
+  <si>
+    <t>V406.nsk_kinetic_model._te.k_7ii = x</t>
+  </si>
+  <si>
+    <t>V406.nsk_kinetic_model._te.k_8 = x</t>
+  </si>
+  <si>
+    <t>V406.nsk_kinetic_model._te.k_9 = x</t>
+  </si>
+  <si>
+    <t>V406.nsk_kinetic_model._te.k_9e = x</t>
+  </si>
+  <si>
+    <t>V406.nsk_kinetic_model._te.k_9c = x</t>
+  </si>
+  <si>
+    <t>V406.nsk_kinetic_model._te.k_10 = x</t>
+  </si>
+  <si>
+    <t>V406.nsk_kinetic_model._te.k_11 = x</t>
   </si>
   <si>
     <t>lime.price = x</t>
@@ -299,55 +299,55 @@
     <t>sulfuric_acid.price = x</t>
   </si>
   <si>
-    <t>V406.kinetic_reaction_system._te.K_1l = x</t>
-  </si>
-  <si>
-    <t>V406.kinetic_reaction_system._te.K_1h = x</t>
-  </si>
-  <si>
-    <t>V406.kinetic_reaction_system._te.K_1i = x</t>
-  </si>
-  <si>
-    <t>V406.kinetic_reaction_system._te.K_1e = x</t>
-  </si>
-  <si>
-    <t>V406.kinetic_reaction_system._te.K_2 = x</t>
-  </si>
-  <si>
-    <t>V406.kinetic_reaction_system._te.K_2i = x</t>
-  </si>
-  <si>
-    <t>V406.kinetic_reaction_system._te.K_3 = x</t>
-  </si>
-  <si>
-    <t>V406.kinetic_reaction_system._te.K_4 = x</t>
-  </si>
-  <si>
-    <t>V406.kinetic_reaction_system._te.K_5 = x</t>
-  </si>
-  <si>
-    <t>V406.kinetic_reaction_system._te.K_5e = x</t>
-  </si>
-  <si>
-    <t>V406.kinetic_reaction_system._te.K_5i = x</t>
-  </si>
-  <si>
-    <t>V406.kinetic_reaction_system._te.K_6 = x</t>
-  </si>
-  <si>
-    <t>V406.kinetic_reaction_system._te.K_6e = x</t>
-  </si>
-  <si>
-    <t>V406.kinetic_reaction_system._te.K_7 = x</t>
-  </si>
-  <si>
-    <t>V406.kinetic_reaction_system._te.K_9 = x</t>
-  </si>
-  <si>
-    <t>V406.kinetic_reaction_system._te.K_9e = x</t>
-  </si>
-  <si>
-    <t>V406.kinetic_reaction_system._te.K_9i = x</t>
+    <t>V406.nsk_kinetic_model._te.K_1l = x</t>
+  </si>
+  <si>
+    <t>V406.nsk_kinetic_model._te.K_1h = x</t>
+  </si>
+  <si>
+    <t>V406.nsk_kinetic_model._te.K_1i = x</t>
+  </si>
+  <si>
+    <t>V406.nsk_kinetic_model._te.K_1e = x</t>
+  </si>
+  <si>
+    <t>V406.nsk_kinetic_model._te.K_2 = x</t>
+  </si>
+  <si>
+    <t>V406.nsk_kinetic_model._te.K_2i = x</t>
+  </si>
+  <si>
+    <t>V406.nsk_kinetic_model._te.K_3 = x</t>
+  </si>
+  <si>
+    <t>V406.nsk_kinetic_model._te.K_4 = x</t>
+  </si>
+  <si>
+    <t>V406.nsk_kinetic_model._te.K_5 = x</t>
+  </si>
+  <si>
+    <t>V406.nsk_kinetic_model._te.K_5e = x</t>
+  </si>
+  <si>
+    <t>V406.nsk_kinetic_model._te.K_5i = x</t>
+  </si>
+  <si>
+    <t>V406.nsk_kinetic_model._te.K_6 = x</t>
+  </si>
+  <si>
+    <t>V406.nsk_kinetic_model._te.K_6e = x</t>
+  </si>
+  <si>
+    <t>V406.nsk_kinetic_model._te.K_7 = x</t>
+  </si>
+  <si>
+    <t>V406.nsk_kinetic_model._te.K_9 = x</t>
+  </si>
+  <si>
+    <t>V406.nsk_kinetic_model._te.K_9e = x</t>
+  </si>
+  <si>
+    <t>V406.nsk_kinetic_model._te.K_9i = x</t>
   </si>
   <si>
     <t>K_1l</t>

</xml_diff>